<commit_message>
fix: distribute dynamic challenge criteria across Alola progression
Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Alola_Paths_and_Challenges.xlsx
+++ b/Alola_Paths_and_Challenges.xlsx
@@ -435,7 +435,7 @@
         <v>Pikipek</v>
       </c>
       <c r="E2" t="str">
-        <v>3-8</v>
+        <v>2-7</v>
       </c>
       <c r="F2" t="str">
         <v>12.50%</v>
@@ -455,7 +455,7 @@
         <v>Yungoos</v>
       </c>
       <c r="E3" t="str">
-        <v>3-8</v>
+        <v>2-7</v>
       </c>
       <c r="F3" t="str">
         <v>12.50%</v>
@@ -475,7 +475,7 @@
         <v>Alolan Rattata</v>
       </c>
       <c r="E4" t="str">
-        <v>3-8</v>
+        <v>2-7</v>
       </c>
       <c r="F4" t="str">
         <v>12.50%</v>
@@ -495,7 +495,7 @@
         <v>Ledyba</v>
       </c>
       <c r="E5" t="str">
-        <v>3-8</v>
+        <v>2-7</v>
       </c>
       <c r="F5" t="str">
         <v>12.50%</v>
@@ -515,7 +515,7 @@
         <v>Spinarak</v>
       </c>
       <c r="E6" t="str">
-        <v>3-8</v>
+        <v>2-7</v>
       </c>
       <c r="F6" t="str">
         <v>12.50%</v>
@@ -535,7 +535,7 @@
         <v>Grubbin</v>
       </c>
       <c r="E7" t="str">
-        <v>3-8</v>
+        <v>2-7</v>
       </c>
       <c r="F7" t="str">
         <v>12.50%</v>
@@ -555,7 +555,7 @@
         <v>Pichu</v>
       </c>
       <c r="E8" t="str">
-        <v>3-8</v>
+        <v>2-7</v>
       </c>
       <c r="F8" t="str">
         <v>12.50%</v>
@@ -575,7 +575,7 @@
         <v>Pikachu</v>
       </c>
       <c r="E9" t="str">
-        <v>3-8</v>
+        <v>2-7</v>
       </c>
       <c r="F9" t="str">
         <v>12.50%</v>
@@ -595,7 +595,7 @@
         <v>Inkay</v>
       </c>
       <c r="E10" t="str">
-        <v>5-10</v>
+        <v>3-8</v>
       </c>
       <c r="F10" t="str">
         <v>20.00%</v>
@@ -615,7 +615,7 @@
         <v>Slowpoke</v>
       </c>
       <c r="E11" t="str">
-        <v>5-10</v>
+        <v>3-8</v>
       </c>
       <c r="F11" t="str">
         <v>20.00%</v>
@@ -635,7 +635,7 @@
         <v>Alolan Meowth</v>
       </c>
       <c r="E12" t="str">
-        <v>5-10</v>
+        <v>3-8</v>
       </c>
       <c r="F12" t="str">
         <v>20.00%</v>
@@ -655,7 +655,7 @@
         <v>Tentacool</v>
       </c>
       <c r="E13" t="str">
-        <v>5-10</v>
+        <v>3-8</v>
       </c>
       <c r="F13" t="str">
         <v>20.00%</v>
@@ -675,7 +675,7 @@
         <v>Finneon</v>
       </c>
       <c r="E14" t="str">
-        <v>5-10</v>
+        <v>3-8</v>
       </c>
       <c r="F14" t="str">
         <v>20.00%</v>
@@ -695,7 +695,7 @@
         <v>Furfrou</v>
       </c>
       <c r="E15" t="str">
-        <v>6-11</v>
+        <v>5-10</v>
       </c>
       <c r="F15" t="str">
         <v>20.00%</v>
@@ -715,7 +715,7 @@
         <v>Hypno</v>
       </c>
       <c r="E16" t="str">
-        <v>6-11</v>
+        <v>5-10</v>
       </c>
       <c r="F16" t="str">
         <v>20.00%</v>
@@ -735,7 +735,7 @@
         <v>Abra</v>
       </c>
       <c r="E17" t="str">
-        <v>6-11</v>
+        <v>5-10</v>
       </c>
       <c r="F17" t="str">
         <v>20.00%</v>
@@ -755,7 +755,7 @@
         <v>Mime Jr.</v>
       </c>
       <c r="E18" t="str">
-        <v>6-11</v>
+        <v>5-10</v>
       </c>
       <c r="F18" t="str">
         <v>20.00%</v>
@@ -775,7 +775,7 @@
         <v>Bewear</v>
       </c>
       <c r="E19" t="str">
-        <v>6-11</v>
+        <v>5-10</v>
       </c>
       <c r="F19" t="str">
         <v>20.00%</v>
@@ -795,7 +795,7 @@
         <v>Drowzee</v>
       </c>
       <c r="E20" t="str">
-        <v>8-13</v>
+        <v>6-11</v>
       </c>
       <c r="F20" t="str">
         <v>16.67%</v>
@@ -815,7 +815,7 @@
         <v>Makuhita</v>
       </c>
       <c r="E21" t="str">
-        <v>8-13</v>
+        <v>6-11</v>
       </c>
       <c r="F21" t="str">
         <v>16.67%</v>
@@ -835,7 +835,7 @@
         <v>Spearow</v>
       </c>
       <c r="E22" t="str">
-        <v>8-13</v>
+        <v>6-11</v>
       </c>
       <c r="F22" t="str">
         <v>16.67%</v>
@@ -855,7 +855,7 @@
         <v>Ekans</v>
       </c>
       <c r="E23" t="str">
-        <v>8-13</v>
+        <v>6-11</v>
       </c>
       <c r="F23" t="str">
         <v>16.67%</v>
@@ -875,7 +875,7 @@
         <v>Growlithe</v>
       </c>
       <c r="E24" t="str">
-        <v>8-13</v>
+        <v>6-11</v>
       </c>
       <c r="F24" t="str">
         <v>16.67%</v>
@@ -895,7 +895,7 @@
         <v>Smeargle</v>
       </c>
       <c r="E25" t="str">
-        <v>8-13</v>
+        <v>6-11</v>
       </c>
       <c r="F25" t="str">
         <v>16.67%</v>
@@ -915,7 +915,7 @@
         <v>Boss</v>
       </c>
       <c r="E26" t="str">
-        <v>9-14</v>
+        <v>8-13</v>
       </c>
       <c r="F26" t="str">
         <v>-</v>
@@ -935,7 +935,7 @@
         <v>Gastly</v>
       </c>
       <c r="E27" t="str">
-        <v>11-16</v>
+        <v>9-14</v>
       </c>
       <c r="F27" t="str">
         <v>25.00%</v>
@@ -955,7 +955,7 @@
         <v>Drifloon</v>
       </c>
       <c r="E28" t="str">
-        <v>11-16</v>
+        <v>9-14</v>
       </c>
       <c r="F28" t="str">
         <v>25.00%</v>
@@ -975,7 +975,7 @@
         <v>Murkrow</v>
       </c>
       <c r="E29" t="str">
-        <v>11-16</v>
+        <v>9-14</v>
       </c>
       <c r="F29" t="str">
         <v>25.00%</v>
@@ -995,7 +995,7 @@
         <v>Misdreavus</v>
       </c>
       <c r="E30" t="str">
-        <v>11-16</v>
+        <v>9-14</v>
       </c>
       <c r="F30" t="str">
         <v>25.00%</v>
@@ -1015,7 +1015,7 @@
         <v>Roggenrola</v>
       </c>
       <c r="E31" t="str">
-        <v>15-20</v>
+        <v>14-19</v>
       </c>
       <c r="F31" t="str">
         <v>20.00%</v>
@@ -1035,7 +1035,7 @@
         <v>Carbink</v>
       </c>
       <c r="E32" t="str">
-        <v>15-20</v>
+        <v>14-19</v>
       </c>
       <c r="F32" t="str">
         <v>20.00%</v>
@@ -1055,7 +1055,7 @@
         <v>Spinda</v>
       </c>
       <c r="E33" t="str">
-        <v>15-20</v>
+        <v>14-19</v>
       </c>
       <c r="F33" t="str">
         <v>20.00%</v>
@@ -1075,7 +1075,7 @@
         <v>Mawile</v>
       </c>
       <c r="E34" t="str">
-        <v>15-20</v>
+        <v>14-19</v>
       </c>
       <c r="F34" t="str">
         <v>20.00%</v>
@@ -1095,7 +1095,7 @@
         <v>Lycanroc</v>
       </c>
       <c r="E35" t="str">
-        <v>15-20</v>
+        <v>14-19</v>
       </c>
       <c r="F35" t="str">
         <v>20.00%</v>
@@ -1115,7 +1115,7 @@
         <v>Barboach</v>
       </c>
       <c r="E36" t="str">
-        <v>17-22</v>
+        <v>15-20</v>
       </c>
       <c r="F36" t="str">
         <v>33.33%</v>
@@ -1135,7 +1135,7 @@
         <v>Smoochum</v>
       </c>
       <c r="E37" t="str">
-        <v>17-22</v>
+        <v>15-20</v>
       </c>
       <c r="F37" t="str">
         <v>33.33%</v>
@@ -1155,7 +1155,7 @@
         <v>Seel</v>
       </c>
       <c r="E38" t="str">
-        <v>17-22</v>
+        <v>15-20</v>
       </c>
       <c r="F38" t="str">
         <v>33.33%</v>
@@ -1175,7 +1175,7 @@
         <v>Boss</v>
       </c>
       <c r="E39" t="str">
-        <v>18-23</v>
+        <v>17-22</v>
       </c>
       <c r="F39" t="str">
         <v>-</v>
@@ -1195,7 +1195,7 @@
         <v>Vikavolt</v>
       </c>
       <c r="E40" t="str">
-        <v>20-25</v>
+        <v>18-23</v>
       </c>
       <c r="F40" t="str">
         <v>20.00%</v>
@@ -1215,7 +1215,7 @@
         <v>Ribombee</v>
       </c>
       <c r="E41" t="str">
-        <v>20-25</v>
+        <v>18-23</v>
       </c>
       <c r="F41" t="str">
         <v>20.00%</v>
@@ -1235,7 +1235,7 @@
         <v>Araquanid</v>
       </c>
       <c r="E42" t="str">
-        <v>20-25</v>
+        <v>18-23</v>
       </c>
       <c r="F42" t="str">
         <v>20.00%</v>
@@ -1255,7 +1255,7 @@
         <v>Lurantis</v>
       </c>
       <c r="E43" t="str">
-        <v>20-25</v>
+        <v>18-23</v>
       </c>
       <c r="F43" t="str">
         <v>20.00%</v>
@@ -1275,7 +1275,7 @@
         <v>Salazzle</v>
       </c>
       <c r="E44" t="str">
-        <v>20-25</v>
+        <v>18-23</v>
       </c>
       <c r="F44" t="str">
         <v>20.00%</v>
@@ -1295,7 +1295,7 @@
         <v>Alolan Marowak</v>
       </c>
       <c r="E45" t="str">
-        <v>20-25</v>
+        <v>18-23</v>
       </c>
       <c r="F45" t="str">
         <v>20.00%</v>
@@ -1315,7 +1315,7 @@
         <v>Kommo-o</v>
       </c>
       <c r="E46" t="str">
-        <v>20-25</v>
+        <v>18-23</v>
       </c>
       <c r="F46" t="str">
         <v>20.00%</v>
@@ -1335,7 +1335,7 @@
         <v>Mimikyu</v>
       </c>
       <c r="E47" t="str">
-        <v>20-25</v>
+        <v>18-23</v>
       </c>
       <c r="F47" t="str">
         <v>20.00%</v>
@@ -1355,7 +1355,7 @@
         <v>Poliwhirl</v>
       </c>
       <c r="E48" t="str">
-        <v>20-25</v>
+        <v>18-23</v>
       </c>
       <c r="F48" t="str">
         <v>20.00%</v>
@@ -1375,7 +1375,7 @@
         <v>Ditto</v>
       </c>
       <c r="E49" t="str">
-        <v>20-25</v>
+        <v>18-23</v>
       </c>
       <c r="F49" t="str">
         <v>20.00%</v>
@@ -1395,7 +1395,7 @@
         <v>Eevee</v>
       </c>
       <c r="E50" t="str">
-        <v>21-26</v>
+        <v>20-25</v>
       </c>
       <c r="F50" t="str">
         <v>25.00%</v>
@@ -1415,7 +1415,7 @@
         <v>Mareep</v>
       </c>
       <c r="E51" t="str">
-        <v>21-26</v>
+        <v>20-25</v>
       </c>
       <c r="F51" t="str">
         <v>25.00%</v>
@@ -1435,7 +1435,7 @@
         <v>Tauros</v>
       </c>
       <c r="E52" t="str">
-        <v>21-26</v>
+        <v>20-25</v>
       </c>
       <c r="F52" t="str">
         <v>25.00%</v>
@@ -1455,7 +1455,7 @@
         <v>Miltank</v>
       </c>
       <c r="E53" t="str">
-        <v>21-26</v>
+        <v>20-25</v>
       </c>
       <c r="F53" t="str">
         <v>25.00%</v>
@@ -1495,7 +1495,7 @@
         <v>Noibat</v>
       </c>
       <c r="E55" t="str">
-        <v>24-29</v>
+        <v>23-28</v>
       </c>
       <c r="F55" t="str">
         <v>33.33%</v>
@@ -1515,7 +1515,7 @@
         <v>Fomantis</v>
       </c>
       <c r="E56" t="str">
-        <v>24-29</v>
+        <v>23-28</v>
       </c>
       <c r="F56" t="str">
         <v>33.33%</v>
@@ -1535,7 +1535,7 @@
         <v>Bounsweet</v>
       </c>
       <c r="E57" t="str">
-        <v>24-29</v>
+        <v>23-28</v>
       </c>
       <c r="F57" t="str">
         <v>33.33%</v>
@@ -1555,7 +1555,7 @@
         <v>Wingull</v>
       </c>
       <c r="E58" t="str">
-        <v>25-30</v>
+        <v>24-29</v>
       </c>
       <c r="F58" t="str">
         <v>20.00%</v>
@@ -1575,7 +1575,7 @@
         <v>Lillipup</v>
       </c>
       <c r="E59" t="str">
-        <v>25-30</v>
+        <v>24-29</v>
       </c>
       <c r="F59" t="str">
         <v>20.00%</v>
@@ -1595,7 +1595,7 @@
         <v>Paras</v>
       </c>
       <c r="E60" t="str">
-        <v>25-30</v>
+        <v>24-29</v>
       </c>
       <c r="F60" t="str">
         <v>20.00%</v>
@@ -1615,7 +1615,7 @@
         <v>Goldeen</v>
       </c>
       <c r="E61" t="str">
-        <v>25-30</v>
+        <v>24-29</v>
       </c>
       <c r="F61" t="str">
         <v>20.00%</v>
@@ -1635,7 +1635,7 @@
         <v>Feebas</v>
       </c>
       <c r="E62" t="str">
-        <v>25-30</v>
+        <v>24-29</v>
       </c>
       <c r="F62" t="str">
         <v>20.00%</v>
@@ -1655,7 +1655,7 @@
         <v>Boss</v>
       </c>
       <c r="E63" t="str">
-        <v>27-32</v>
+        <v>26-31</v>
       </c>
       <c r="F63" t="str">
         <v>-</v>
@@ -1675,7 +1675,7 @@
         <v>Cubone</v>
       </c>
       <c r="E64" t="str">
-        <v>28-33</v>
+        <v>27-32</v>
       </c>
       <c r="F64" t="str">
         <v>33.33%</v>
@@ -1695,7 +1695,7 @@
         <v>Kangaskhan</v>
       </c>
       <c r="E65" t="str">
-        <v>28-33</v>
+        <v>27-32</v>
       </c>
       <c r="F65" t="str">
         <v>33.33%</v>
@@ -1715,7 +1715,7 @@
         <v>Magby</v>
       </c>
       <c r="E66" t="str">
-        <v>28-33</v>
+        <v>27-32</v>
       </c>
       <c r="F66" t="str">
         <v>33.33%</v>
@@ -1735,7 +1735,7 @@
         <v>Boss</v>
       </c>
       <c r="E67" t="str">
-        <v>30-35</v>
+        <v>29-34</v>
       </c>
       <c r="F67" t="str">
         <v>-</v>
@@ -1755,7 +1755,7 @@
         <v>Staryu</v>
       </c>
       <c r="E68" t="str">
-        <v>31-36</v>
+        <v>30-35</v>
       </c>
       <c r="F68" t="str">
         <v>20.00%</v>
@@ -1775,7 +1775,7 @@
         <v>Pyukumuku</v>
       </c>
       <c r="E69" t="str">
-        <v>31-36</v>
+        <v>30-35</v>
       </c>
       <c r="F69" t="str">
         <v>20.00%</v>
@@ -1795,7 +1795,7 @@
         <v>Corsola</v>
       </c>
       <c r="E70" t="str">
-        <v>31-36</v>
+        <v>30-35</v>
       </c>
       <c r="F70" t="str">
         <v>20.00%</v>
@@ -1815,7 +1815,7 @@
         <v>Mareanie</v>
       </c>
       <c r="E71" t="str">
-        <v>31-36</v>
+        <v>30-35</v>
       </c>
       <c r="F71" t="str">
         <v>20.00%</v>
@@ -1835,7 +1835,7 @@
         <v>Bruxish</v>
       </c>
       <c r="E72" t="str">
-        <v>31-36</v>
+        <v>30-35</v>
       </c>
       <c r="F72" t="str">
         <v>20.00%</v>
@@ -1855,7 +1855,7 @@
         <v>Omanyte</v>
       </c>
       <c r="E73" t="str">
-        <v>33-38</v>
+        <v>32-37</v>
       </c>
       <c r="F73" t="str">
         <v>20.00%</v>
@@ -1875,7 +1875,7 @@
         <v>Kabuto</v>
       </c>
       <c r="E74" t="str">
-        <v>33-38</v>
+        <v>32-37</v>
       </c>
       <c r="F74" t="str">
         <v>20.00%</v>
@@ -1895,7 +1895,7 @@
         <v>Lileep</v>
       </c>
       <c r="E75" t="str">
-        <v>33-38</v>
+        <v>32-37</v>
       </c>
       <c r="F75" t="str">
         <v>20.00%</v>
@@ -1915,7 +1915,7 @@
         <v>Anorith</v>
       </c>
       <c r="E76" t="str">
-        <v>33-38</v>
+        <v>32-37</v>
       </c>
       <c r="F76" t="str">
         <v>20.00%</v>
@@ -1935,7 +1935,7 @@
         <v>Cranidos</v>
       </c>
       <c r="E77" t="str">
-        <v>33-38</v>
+        <v>32-37</v>
       </c>
       <c r="F77" t="str">
         <v>20.00%</v>
@@ -1955,7 +1955,7 @@
         <v>Shieldon</v>
       </c>
       <c r="E78" t="str">
-        <v>33-38</v>
+        <v>32-37</v>
       </c>
       <c r="F78" t="str">
         <v>20.00%</v>
@@ -1975,7 +1975,7 @@
         <v>Archen</v>
       </c>
       <c r="E79" t="str">
-        <v>33-38</v>
+        <v>32-37</v>
       </c>
       <c r="F79" t="str">
         <v>20.00%</v>
@@ -1995,7 +1995,7 @@
         <v>Tirtouga</v>
       </c>
       <c r="E80" t="str">
-        <v>33-38</v>
+        <v>32-37</v>
       </c>
       <c r="F80" t="str">
         <v>20.00%</v>
@@ -2015,7 +2015,7 @@
         <v>Tyrunt</v>
       </c>
       <c r="E81" t="str">
-        <v>33-38</v>
+        <v>32-37</v>
       </c>
       <c r="F81" t="str">
         <v>20.00%</v>
@@ -2035,7 +2035,7 @@
         <v>Amaura</v>
       </c>
       <c r="E82" t="str">
-        <v>33-38</v>
+        <v>32-37</v>
       </c>
       <c r="F82" t="str">
         <v>20.00%</v>
@@ -2055,7 +2055,7 @@
         <v>Trumbeak</v>
       </c>
       <c r="E83" t="str">
-        <v>34-39</v>
+        <v>33-38</v>
       </c>
       <c r="F83" t="str">
         <v>16.67%</v>
@@ -2075,7 +2075,7 @@
         <v>Steenee</v>
       </c>
       <c r="E84" t="str">
-        <v>34-39</v>
+        <v>33-38</v>
       </c>
       <c r="F84" t="str">
         <v>16.67%</v>
@@ -2095,7 +2095,7 @@
         <v>Comfey</v>
       </c>
       <c r="E85" t="str">
-        <v>34-39</v>
+        <v>33-38</v>
       </c>
       <c r="F85" t="str">
         <v>16.67%</v>
@@ -2115,7 +2115,7 @@
         <v>Hoothoot</v>
       </c>
       <c r="E86" t="str">
-        <v>34-39</v>
+        <v>33-38</v>
       </c>
       <c r="F86" t="str">
         <v>16.67%</v>
@@ -2135,7 +2135,7 @@
         <v>Oranguru</v>
       </c>
       <c r="E87" t="str">
-        <v>34-39</v>
+        <v>33-38</v>
       </c>
       <c r="F87" t="str">
         <v>16.67%</v>
@@ -2155,7 +2155,7 @@
         <v>Bounsweet</v>
       </c>
       <c r="E88" t="str">
-        <v>34-39</v>
+        <v>33-38</v>
       </c>
       <c r="F88" t="str">
         <v>16.67%</v>
@@ -2175,7 +2175,7 @@
         <v>Golbat</v>
       </c>
       <c r="E89" t="str">
-        <v>36-41</v>
+        <v>35-40</v>
       </c>
       <c r="F89" t="str">
         <v>20.00%</v>
@@ -2195,7 +2195,7 @@
         <v>Salandit</v>
       </c>
       <c r="E90" t="str">
-        <v>36-41</v>
+        <v>35-40</v>
       </c>
       <c r="F90" t="str">
         <v>20.00%</v>
@@ -2215,7 +2215,7 @@
         <v>Larvesta</v>
       </c>
       <c r="E91" t="str">
-        <v>36-41</v>
+        <v>35-40</v>
       </c>
       <c r="F91" t="str">
         <v>20.00%</v>
@@ -2235,7 +2235,7 @@
         <v>Oranguru</v>
       </c>
       <c r="E92" t="str">
-        <v>36-41</v>
+        <v>35-40</v>
       </c>
       <c r="F92" t="str">
         <v>20.00%</v>
@@ -2255,7 +2255,7 @@
         <v>Passimian</v>
       </c>
       <c r="E93" t="str">
-        <v>36-41</v>
+        <v>35-40</v>
       </c>
       <c r="F93" t="str">
         <v>20.00%</v>
@@ -2275,7 +2275,7 @@
         <v>Boss</v>
       </c>
       <c r="E94" t="str">
-        <v>37-42</v>
+        <v>36-41</v>
       </c>
       <c r="F94" t="str">
         <v>-</v>
@@ -2295,7 +2295,7 @@
         <v>Zubat</v>
       </c>
       <c r="E95" t="str">
-        <v>39-44</v>
+        <v>38-43</v>
       </c>
       <c r="F95" t="str">
         <v>25.00%</v>
@@ -2315,7 +2315,7 @@
         <v>Alolan Diglett</v>
       </c>
       <c r="E96" t="str">
-        <v>39-44</v>
+        <v>38-43</v>
       </c>
       <c r="F96" t="str">
         <v>25.00%</v>
@@ -2335,7 +2335,7 @@
         <v>Kecleon</v>
       </c>
       <c r="E97" t="str">
-        <v>39-44</v>
+        <v>38-43</v>
       </c>
       <c r="F97" t="str">
         <v>25.00%</v>
@@ -2355,7 +2355,7 @@
         <v>Larvitar</v>
       </c>
       <c r="E98" t="str">
-        <v>39-44</v>
+        <v>38-43</v>
       </c>
       <c r="F98" t="str">
         <v>25.00%</v>
@@ -2375,7 +2375,7 @@
         <v>Gumshoos</v>
       </c>
       <c r="E99" t="str">
-        <v>43-48</v>
+        <v>42-47</v>
       </c>
       <c r="F99" t="str">
         <v>12.50%</v>
@@ -2395,7 +2395,7 @@
         <v>Wingull</v>
       </c>
       <c r="E100" t="str">
-        <v>43-48</v>
+        <v>42-47</v>
       </c>
       <c r="F100" t="str">
         <v>12.50%</v>
@@ -2415,7 +2415,7 @@
         <v>Magikarp</v>
       </c>
       <c r="E101" t="str">
-        <v>43-48</v>
+        <v>42-47</v>
       </c>
       <c r="F101" t="str">
         <v>12.50%</v>
@@ -2435,7 +2435,7 @@
         <v>Stufful</v>
       </c>
       <c r="E102" t="str">
-        <v>43-48</v>
+        <v>42-47</v>
       </c>
       <c r="F102" t="str">
         <v>12.50%</v>
@@ -2455,7 +2455,7 @@
         <v>Chinchou</v>
       </c>
       <c r="E103" t="str">
-        <v>43-48</v>
+        <v>42-47</v>
       </c>
       <c r="F103" t="str">
         <v>12.50%</v>
@@ -2475,7 +2475,7 @@
         <v>Alolan Raticate</v>
       </c>
       <c r="E104" t="str">
-        <v>43-48</v>
+        <v>42-47</v>
       </c>
       <c r="F104" t="str">
         <v>12.50%</v>
@@ -2495,7 +2495,7 @@
         <v>Natu</v>
       </c>
       <c r="E105" t="str">
-        <v>43-48</v>
+        <v>42-47</v>
       </c>
       <c r="F105" t="str">
         <v>12.50%</v>
@@ -2515,7 +2515,7 @@
         <v>Nosepass</v>
       </c>
       <c r="E106" t="str">
-        <v>43-48</v>
+        <v>42-47</v>
       </c>
       <c r="F106" t="str">
         <v>12.50%</v>
@@ -2775,7 +2775,7 @@
         <v>Cleffa</v>
       </c>
       <c r="E119" t="str">
-        <v>52-57</v>
+        <v>51-56</v>
       </c>
       <c r="F119" t="str">
         <v>25.00%</v>
@@ -2795,7 +2795,7 @@
         <v>Elgyem</v>
       </c>
       <c r="E120" t="str">
-        <v>52-57</v>
+        <v>51-56</v>
       </c>
       <c r="F120" t="str">
         <v>25.00%</v>
@@ -2815,7 +2815,7 @@
         <v>Beldum</v>
       </c>
       <c r="E121" t="str">
-        <v>52-57</v>
+        <v>51-56</v>
       </c>
       <c r="F121" t="str">
         <v>25.00%</v>
@@ -2835,7 +2835,7 @@
         <v>Minior</v>
       </c>
       <c r="E122" t="str">
-        <v>52-57</v>
+        <v>51-56</v>
       </c>
       <c r="F122" t="str">
         <v>25.00%</v>
@@ -2875,7 +2875,7 @@
         <v>Shiinotic</v>
       </c>
       <c r="E124" t="str">
-        <v>55-60</v>
+        <v>54-59</v>
       </c>
       <c r="F124" t="str">
         <v>11.11%</v>
@@ -2895,7 +2895,7 @@
         <v>Parasect</v>
       </c>
       <c r="E125" t="str">
-        <v>55-60</v>
+        <v>54-59</v>
       </c>
       <c r="F125" t="str">
         <v>11.11%</v>
@@ -2915,7 +2915,7 @@
         <v>Komala</v>
       </c>
       <c r="E126" t="str">
-        <v>55-60</v>
+        <v>54-59</v>
       </c>
       <c r="F126" t="str">
         <v>11.11%</v>
@@ -2935,7 +2935,7 @@
         <v>Houndoom</v>
       </c>
       <c r="E127" t="str">
-        <v>55-60</v>
+        <v>54-59</v>
       </c>
       <c r="F127" t="str">
         <v>11.11%</v>
@@ -2955,7 +2955,7 @@
         <v>Manectric</v>
       </c>
       <c r="E128" t="str">
-        <v>55-60</v>
+        <v>54-59</v>
       </c>
       <c r="F128" t="str">
         <v>11.11%</v>
@@ -2975,7 +2975,7 @@
         <v>Scraggy</v>
       </c>
       <c r="E129" t="str">
-        <v>55-60</v>
+        <v>54-59</v>
       </c>
       <c r="F129" t="str">
         <v>11.11%</v>
@@ -2995,7 +2995,7 @@
         <v>Bisharp</v>
       </c>
       <c r="E130" t="str">
-        <v>55-60</v>
+        <v>54-59</v>
       </c>
       <c r="F130" t="str">
         <v>11.11%</v>
@@ -3015,7 +3015,7 @@
         <v>Machop</v>
       </c>
       <c r="E131" t="str">
-        <v>55-60</v>
+        <v>54-59</v>
       </c>
       <c r="F131" t="str">
         <v>11.11%</v>
@@ -3035,7 +3035,7 @@
         <v>Hawlucha</v>
       </c>
       <c r="E132" t="str">
-        <v>55-60</v>
+        <v>54-59</v>
       </c>
       <c r="F132" t="str">
         <v>11.11%</v>
@@ -3055,7 +3055,7 @@
         <v>Alolan Dugtrio</v>
       </c>
       <c r="E133" t="str">
-        <v>58-63</v>
+        <v>57-62</v>
       </c>
       <c r="F133" t="str">
         <v>20.00%</v>
@@ -3075,7 +3075,7 @@
         <v>Sandile</v>
       </c>
       <c r="E134" t="str">
-        <v>58-63</v>
+        <v>57-62</v>
       </c>
       <c r="F134" t="str">
         <v>20.00%</v>
@@ -3095,7 +3095,7 @@
         <v>Krokorok</v>
       </c>
       <c r="E135" t="str">
-        <v>58-63</v>
+        <v>57-62</v>
       </c>
       <c r="F135" t="str">
         <v>20.00%</v>
@@ -3115,7 +3115,7 @@
         <v>Staryu</v>
       </c>
       <c r="E136" t="str">
-        <v>58-63</v>
+        <v>57-62</v>
       </c>
       <c r="F136" t="str">
         <v>20.00%</v>
@@ -3135,7 +3135,7 @@
         <v>Sandygast</v>
       </c>
       <c r="E137" t="str">
-        <v>58-63</v>
+        <v>57-62</v>
       </c>
       <c r="F137" t="str">
         <v>20.00%</v>
@@ -3355,7 +3355,7 @@
         <v>Boss</v>
       </c>
       <c r="E148" t="str">
-        <v>64-69</v>
+        <v>63-68</v>
       </c>
       <c r="F148" t="str">
         <v>-</v>
@@ -5208,7 +5208,7 @@
         <v>Challenge 1</v>
       </c>
       <c r="B2" t="str">
-        <v>Defeat 10 Pokemon in Route 1 East</v>
+        <v>Defeat 15 Pokemon in Route 1 East</v>
       </c>
       <c r="C2" t="str">
         <v>Unlocks Route 1 Hau'oli Outskirts</v>
@@ -5219,7 +5219,7 @@
         <v>Challenge 2</v>
       </c>
       <c r="B3" t="str">
-        <v>Defeat 10 Pokemon in Route 1 Hau'oli Outskirts</v>
+        <v>Catch 3 Dark type Pokemon in Route 1 Hau'oli Outskirts</v>
       </c>
       <c r="C3" t="str">
         <v>Unlocks Hau'oli City Shopping District</v>
@@ -5230,7 +5230,7 @@
         <v>Challenge 3</v>
       </c>
       <c r="B4" t="str">
-        <v>Defeat 10 Pokemon in Hau'oli City Shopping District</v>
+        <v>Catch 5 Pokemon of Uncommon or better rarity in Hau'oli City Shopping District</v>
       </c>
       <c r="C4" t="str">
         <v>Unlocks Route 2 North</v>
@@ -5241,7 +5241,7 @@
         <v>Challenge 4</v>
       </c>
       <c r="B5" t="str">
-        <v>Defeat 10 Pokemon in Route 2 North</v>
+        <v>Catch 2 Pokemon of Rare or better rarity in Route 2 North</v>
       </c>
       <c r="C5" t="str">
         <v>Unlocks Captain Ilima</v>
@@ -5263,7 +5263,7 @@
         <v>Challenge 6</v>
       </c>
       <c r="B7" t="str">
-        <v>Defeat 10 Pokemon in Hau'oli Cemetery Main Area</v>
+        <v>Catch 1 Epic rarity Pokemon in Hau'oli Cemetery Main Area</v>
       </c>
       <c r="C7" t="str">
         <v>Unlocks Ten Carat Hill Farthest Hollow</v>
@@ -5274,7 +5274,7 @@
         <v>Challenge 7</v>
       </c>
       <c r="B8" t="str">
-        <v>Defeat 10 Pokemon in Ten Carat Hill Farthest Hollow</v>
+        <v>Defeat 5 specific Rock type Pokemon</v>
       </c>
       <c r="C8" t="str">
         <v>Unlocks Seaward Cave Main Area</v>
@@ -5285,7 +5285,7 @@
         <v>Challenge 8</v>
       </c>
       <c r="B9" t="str">
-        <v>Defeat 10 Pokemon in Seaward Cave Main Area</v>
+        <v>Catch 10 Pokemon in Seaward Cave Main Area</v>
       </c>
       <c r="C9" t="str">
         <v>Unlocks Kahuna Hala</v>
@@ -5318,7 +5318,7 @@
         <v>Challenge 11</v>
       </c>
       <c r="B12" t="str">
-        <v>Defeat 10 Pokemon in Heahea Beach Main Area Part 2</v>
+        <v>Defeat 15 Pokemon in Heahea Beach Main Area Part 2</v>
       </c>
       <c r="C12" t="str">
         <v>Unlocks Paniola Ranch Main Area</v>
@@ -5329,7 +5329,7 @@
         <v>Challenge 12</v>
       </c>
       <c r="B13" t="str">
-        <v>Defeat 10 Pokemon in Paniola Ranch Main Area</v>
+        <v>Catch 3 Normal type Pokemon in Paniola Ranch Main Area</v>
       </c>
       <c r="C13" t="str">
         <v>Unlocks Daycare NPC</v>
@@ -5351,7 +5351,7 @@
         <v>Challenge 14</v>
       </c>
       <c r="B15" t="str">
-        <v>Defeat 10 Pokemon in Route 5 Main Area</v>
+        <v>Catch 5 Pokemon of Uncommon or better rarity in Route 5 Main Area</v>
       </c>
       <c r="C15" t="str">
         <v>Unlocks Brooklet Hill South</v>
@@ -5362,7 +5362,7 @@
         <v>Challenge 15</v>
       </c>
       <c r="B16" t="str">
-        <v>Defeat 10 Pokemon in Brooklet Hill South</v>
+        <v>Catch 2 Pokemon of Rare or better rarity in Brooklet Hill South</v>
       </c>
       <c r="C16" t="str">
         <v>Unlocks Captain Lana</v>
@@ -5395,7 +5395,7 @@
         <v>Challenge 18</v>
       </c>
       <c r="B19" t="str">
-        <v>Defeat 10 Pokemon in Route 7 Main Area</v>
+        <v>Defeat 5 specific Water type Pokemon</v>
       </c>
       <c r="C19" t="str">
         <v>Unlocks Route 8 Fossil Restoration Center Part 1</v>
@@ -5406,7 +5406,7 @@
         <v>Challenge 19</v>
       </c>
       <c r="B20" t="str">
-        <v>Defeat 10 Pokemon in Route 8 Fossil Restoration Center Part 1</v>
+        <v>Catch 10 Pokemon in Route 8 Fossil Restoration Center Part 1</v>
       </c>
       <c r="C20" t="str">
         <v>Unlocks Route 8 Fossil Restoration Center Part 2</v>
@@ -5417,7 +5417,7 @@
         <v>Challenge 20</v>
       </c>
       <c r="B21" t="str">
-        <v>Defeat 10 Pokemon in Route 8 Fossil Restoration Center Part 2</v>
+        <v>Catch 2 specific Pokemon species in Route 8 Fossil Restoration Center Part 2</v>
       </c>
       <c r="C21" t="str">
         <v>Unlocks Lush Jungle North</v>
@@ -5428,7 +5428,7 @@
         <v>Challenge 21</v>
       </c>
       <c r="B22" t="str">
-        <v>Defeat 10 Pokemon in Lush Jungle North</v>
+        <v>Defeat 15 Pokemon in Lush Jungle North</v>
       </c>
       <c r="C22" t="str">
         <v>Unlocks Lush Jungle East Cave</v>
@@ -5439,7 +5439,7 @@
         <v>Challenge 22</v>
       </c>
       <c r="B23" t="str">
-        <v>Defeat 10 Pokemon in Lush Jungle East Cave</v>
+        <v>Catch 3 Poison type Pokemon in Lush Jungle East Cave</v>
       </c>
       <c r="C23" t="str">
         <v>Unlocks Captain Mallow</v>
@@ -5461,7 +5461,7 @@
         <v>Challenge 24</v>
       </c>
       <c r="B25" t="str">
-        <v>Defeat 10 Pokemon in Diglett's Tunnel Main Area</v>
+        <v>Catch 5 Pokemon of Uncommon or better rarity in Diglett's Tunnel Main Area</v>
       </c>
       <c r="C25" t="str">
         <v>Unlocks Akala Outskirts Main Area</v>
@@ -5472,7 +5472,7 @@
         <v>Challenge 25</v>
       </c>
       <c r="B26" t="str">
-        <v>Defeat 10 Pokemon in Akala Outskirts Main Area</v>
+        <v>Catch 2 Pokemon of Rare or better rarity in Akala Outskirts Main Area</v>
       </c>
       <c r="C26" t="str">
         <v>Unlocks Kahuna Olivia</v>
@@ -5494,7 +5494,7 @@
         <v>Challenge 27</v>
       </c>
       <c r="B28" t="str">
-        <v>Defeat 10 Pokemon in Malie City Outer Cape</v>
+        <v>Catch 1 Epic rarity Pokemon in Malie City Outer Cape</v>
       </c>
       <c r="C28" t="str">
         <v>Unlocks Route 10 Main Area</v>
@@ -5505,7 +5505,7 @@
         <v>Challenge 28</v>
       </c>
       <c r="B29" t="str">
-        <v>Defeat 10 Pokemon in Route 10 Main Area</v>
+        <v>Defeat 5 specific Bug type Pokemon</v>
       </c>
       <c r="C29" t="str">
         <v>Unlocks Mount Hokulani East</v>
@@ -5516,7 +5516,7 @@
         <v>Challenge 29</v>
       </c>
       <c r="B30" t="str">
-        <v>Defeat 10 Pokemon in Mount Hokulani East</v>
+        <v>Catch 10 Pokemon in Mount Hokulani East</v>
       </c>
       <c r="C30" t="str">
         <v>Unlocks Captain Sophocles</v>
@@ -5538,7 +5538,7 @@
         <v>Challenge 31</v>
       </c>
       <c r="B32" t="str">
-        <v>Defeat 10 Pokemon in Route 11 Main Area</v>
+        <v>Catch 2 specific Pokemon species in Route 11 Main Area</v>
       </c>
       <c r="C32" t="str">
         <v>Unlocks Haina Desert Main Area</v>
@@ -5549,7 +5549,7 @@
         <v>Challenge 32</v>
       </c>
       <c r="B33" t="str">
-        <v>Defeat 10 Pokemon in Haina Desert Main Area</v>
+        <v>Defeat 15 Pokemon in Haina Desert Main Area</v>
       </c>
       <c r="C33" t="str">
         <v>Unlocks Tapu Village Main Area</v>
@@ -5560,7 +5560,7 @@
         <v>Challenge 33</v>
       </c>
       <c r="B34" t="str">
-        <v>Defeat 10 Pokemon in Tapu Village Main Area</v>
+        <v>Catch 3 Rock type Pokemon in Tapu Village Main Area</v>
       </c>
       <c r="C34" t="str">
         <v>Unlocks Thrifty Megamart Abandoned Site</v>
@@ -5571,7 +5571,7 @@
         <v>Challenge 34</v>
       </c>
       <c r="B35" t="str">
-        <v>Defeat 10 Pokemon in Thrifty Megamart Abandoned Site</v>
+        <v>Catch 5 Pokemon of Uncommon or better rarity in Thrifty Megamart Abandoned Site</v>
       </c>
       <c r="C35" t="str">
         <v>Unlocks Captain Acerola</v>
@@ -5604,7 +5604,7 @@
         <v>Challenge 37</v>
       </c>
       <c r="B38" t="str">
-        <v>Defeat 10 Pokemon in Seafolk Village Main</v>
+        <v>Catch 2 Pokemon of Rare or better rarity in Seafolk Village Main</v>
       </c>
       <c r="C38" t="str">
         <v>Unlocks Poni Wilds Main Area</v>
@@ -5615,7 +5615,7 @@
         <v>Challenge 38</v>
       </c>
       <c r="B39" t="str">
-        <v>Defeat 10 Pokemon in Poni Wilds Main Area</v>
+        <v>Catch 1 Epic rarity Pokemon in Poni Wilds Main Area</v>
       </c>
       <c r="C39" t="str">
         <v>Unlocks Poni Breaker Coast Main Area</v>
@@ -5626,7 +5626,7 @@
         <v>Challenge 39</v>
       </c>
       <c r="B40" t="str">
-        <v>Defeat 10 Pokemon in Poni Breaker Coast Main Area</v>
+        <v>Defeat 5 specific Bug type Pokemon</v>
       </c>
       <c r="C40" t="str">
         <v>Unlocks Exeggutor Island Main Area</v>
@@ -5637,7 +5637,7 @@
         <v>Challenge 40</v>
       </c>
       <c r="B41" t="str">
-        <v>Defeat 10 Pokemon in Exeggutor Island Main Area</v>
+        <v>Catch 10 Pokemon in Exeggutor Island Main Area</v>
       </c>
       <c r="C41" t="str">
         <v>Unlocks Vast Poni Canyon Outside</v>
@@ -5648,7 +5648,7 @@
         <v>Challenge 41</v>
       </c>
       <c r="B42" t="str">
-        <v>Defeat 10 Pokemon in Vast Poni Canyon Outside</v>
+        <v>Catch 2 specific Pokemon species in Vast Poni Canyon Outside</v>
       </c>
       <c r="C42" t="str">
         <v>Unlocks Captain Kommo-o</v>
@@ -5692,7 +5692,7 @@
         <v>Challenge 45</v>
       </c>
       <c r="B46" t="str">
-        <v>Defeat 10 Pokemon in Mount Lanakila Cave</v>
+        <v>Defeat 15 Pokemon in Mount Lanakila Cave</v>
       </c>
       <c r="C46" t="str">
         <v>Unlocks Alola Pokemon League</v>
@@ -5714,7 +5714,7 @@
         <v>Extra Challenge A-1</v>
       </c>
       <c r="B48" t="str">
-        <v>Defeat 15 Pokemon in Route 1 East</v>
+        <v>Defeat Captain Lana</v>
       </c>
       <c r="C48" t="str">
         <v>Unlocks Route 6 Main Area</v>
@@ -5725,7 +5725,7 @@
         <v>Extra Challenge A-2</v>
       </c>
       <c r="B49" t="str">
-        <v>Defeat 15 Pokemon in Route 6 Main Area</v>
+        <v>Defeat 10 Pokemon in Route 6 Main Area</v>
       </c>
       <c r="C49" t="str">
         <v>Unlocks Royal Avenue Main Area</v>
@@ -5736,7 +5736,7 @@
         <v>Extra Challenge A-3</v>
       </c>
       <c r="B50" t="str">
-        <v>Defeat 15 Pokemon in Royal Avenue Main Area</v>
+        <v>Catch 3 Fire type Pokemon in Royal Avenue Main Area</v>
       </c>
       <c r="C50" t="str">
         <v>Unlocks Pikachu Valley Main Area</v>
@@ -5747,7 +5747,7 @@
         <v>Extra Challenge A-4</v>
       </c>
       <c r="B51" t="str">
-        <v>Defeat 15 Pokemon in Pikachu Valley Main Area</v>
+        <v>Catch 5 Pokemon of Uncommon or better rarity in Pikachu Valley Main Area</v>
       </c>
       <c r="C51" t="str">
         <v>Unlocks Starter Depot Main Area</v>
@@ -5769,7 +5769,7 @@
         <v>Extra Challenge B-2</v>
       </c>
       <c r="B53" t="str">
-        <v>Defeat 15 Pokemon in Poni Coast Main Area</v>
+        <v>Catch 2 Pokemon of Rare or better rarity in Poni Coast Main Area</v>
       </c>
       <c r="C53" t="str">
         <v>Unlocks Shopping Mall Antiquities Event</v>
@@ -5780,7 +5780,7 @@
         <v>Extra Challenge B-3</v>
       </c>
       <c r="B54" t="str">
-        <v>Defeat 15 Pokemon in Shopping Mall Antiquities Event</v>
+        <v>Defeat 10 Pokemon in Shopping Mall Antiquities Event</v>
       </c>
       <c r="C54" t="str">
         <v>Unlocks Aether Paradise Restricted Area</v>
@@ -5791,7 +5791,7 @@
         <v>Extra Challenge B-4</v>
       </c>
       <c r="B55" t="str">
-        <v>Defeat 15 Pokemon in Aether Paradise Restricted Area</v>
+        <v>Defeat 10 Pokemon in Aether Paradise Restricted Area</v>
       </c>
       <c r="C55" t="str">
         <v>Unlocks The Zenith Anomaly Main Area</v>
@@ -5813,7 +5813,7 @@
         <v>Extra Challenge C-2</v>
       </c>
       <c r="B57" t="str">
-        <v>Defeat 15 Pokemon in Mahalo Trail Main Area</v>
+        <v>Defeat 10 Pokemon in Mahalo Trail Main Area</v>
       </c>
       <c r="C57" t="str">
         <v>Unlocks Melemele Meadow Main Area</v>
@@ -5824,7 +5824,7 @@
         <v>Extra Challenge C-3</v>
       </c>
       <c r="B58" t="str">
-        <v>Defeat 15 Pokemon in Melemele Meadow Main Area</v>
+        <v>Catch 1 Epic rarity Pokemon in Melemele Meadow Main Area</v>
       </c>
       <c r="C58" t="str">
         <v>Unlocks Ruins of Conflict Special Encounter</v>
@@ -5835,7 +5835,7 @@
         <v>Extra Challenge C-4</v>
       </c>
       <c r="B59" t="str">
-        <v>Defeat 15 Pokemon in Ruins of Conflict Special Encounter</v>
+        <v>Defeat 10 Pokemon in Ruins of Conflict Special Encounter</v>
       </c>
       <c r="C59" t="str">
         <v>Unlocks Memorial Hill Main</v>
@@ -5846,7 +5846,7 @@
         <v>Extra Challenge C-5</v>
       </c>
       <c r="B60" t="str">
-        <v>Defeat 15 Pokemon in Memorial Hill Main</v>
+        <v>Defeat 10 Pokemon in Memorial Hill Main</v>
       </c>
       <c r="C60" t="str">
         <v>Unlocks Sacred Shrine Main Area</v>
@@ -5868,7 +5868,7 @@
         <v>Extra Challenge D-2</v>
       </c>
       <c r="B62" t="str">
-        <v>Defeat 15 Pokemon in Poni Grove Main Area</v>
+        <v>Defeat 5 specific Normal type Pokemon</v>
       </c>
       <c r="C62" t="str">
         <v>Unlocks Poni Plains Center</v>
@@ -5879,7 +5879,7 @@
         <v>Extra Challenge D-3</v>
       </c>
       <c r="B63" t="str">
-        <v>Defeat 15 Pokemon in Poni Plains Center</v>
+        <v>Defeat 10 Pokemon in Poni Plains Center</v>
       </c>
       <c r="C63" t="str">
         <v>Unlocks Resolution Cave Main Area</v>
@@ -5890,7 +5890,7 @@
         <v>Extra Challenge D-4</v>
       </c>
       <c r="B64" t="str">
-        <v>Defeat 15 Pokemon in Resolution Cave Main Area</v>
+        <v>Defeat 10 Pokemon in Resolution Cave Main Area</v>
       </c>
       <c r="C64" t="str">
         <v>Unlocks Ruins of Hope Special Encounter</v>
@@ -5901,7 +5901,7 @@
         <v>Extra Challenge D-5</v>
       </c>
       <c r="B65" t="str">
-        <v>Defeat 15 Pokemon in Ruins of Hope Special Encounter</v>
+        <v>Defeat 10 Pokemon in Ruins of Hope Special Encounter</v>
       </c>
       <c r="C65" t="str">
         <v>Unlocks The Interdimensional Rift Main Area</v>
@@ -5923,7 +5923,7 @@
         <v>Extra Challenge E-2</v>
       </c>
       <c r="B67" t="str">
-        <v>Defeat 15 Pokemon in Route 15 Main Area</v>
+        <v>Defeat 10 Pokemon in Route 15 Main Area</v>
       </c>
       <c r="C67" t="str">
         <v>Unlocks Aether Paradise Labs</v>
@@ -5934,7 +5934,7 @@
         <v>Extra Challenge E-3</v>
       </c>
       <c r="B68" t="str">
-        <v>Defeat 15 Pokemon in Aether Paradise Labs</v>
+        <v>Defeat 10 Pokemon in Aether Paradise Labs</v>
       </c>
       <c r="C68" t="str">
         <v>Unlocks Aether Paradise Secret Lab</v>
@@ -5945,7 +5945,7 @@
         <v>Extra Challenge E-4</v>
       </c>
       <c r="B69" t="str">
-        <v>Defeat 15 Pokemon in Aether Paradise Secret Lab</v>
+        <v>Catch 10 Pokemon in Aether Paradise Secret Lab</v>
       </c>
       <c r="C69" t="str">
         <v>Unlocks Lake of the Sunne Main Area</v>
@@ -5956,7 +5956,7 @@
         <v>Extra Challenge E-5</v>
       </c>
       <c r="B70" t="str">
-        <v>Defeat 15 Pokemon in Lake of the Sunne Main Area</v>
+        <v>Catch 2 specific Pokemon species in Lake of the Sunne Main Area</v>
       </c>
       <c r="C70" t="str">
         <v>Unlocks Obsidian Sphere Main Area</v>

</xml_diff>